<commit_message>
update: monthly data 週一 2026/09/07
</commit_message>
<xml_diff>
--- a/data/AIRSPACE_線下通路_行銷排程_含甘特圖_2025-2026.xlsx
+++ b/data/AIRSPACE_線下通路_行銷排程_含甘特圖_2025-2026.xlsx
@@ -12,12 +12,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">行銷排程!$A$1:$I$151</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1285" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="460">
   <si>
     <t>年度</t>
   </si>
@@ -1288,12 +1288,6 @@
     <t>如消費滿2500且加購手機支架，則KEY入兩個贈品，系統會自動判斷一個為加購價/一個為贈品;請務必確實銷貨，若有漏KEY，可另外成立一單備註補XX單之贈品;贈不織布袋及手機鍊僅販售CA及PLUS及IP店櫃適用活動，贈手機支架全體正價店適用</t>
   </si>
   <si>
-    <t>6/4-6/21</t>
-  </si>
-  <si>
-    <t>2026/06/03郵件</t>
-  </si>
-  <si>
     <t>2026/06/10郵件</t>
   </si>
   <si>
@@ -1321,9 +1315,6 @@
     <t>2026/06/18郵件</t>
   </si>
   <si>
-    <t>8/1起 官網下單門市取貨獨家 凡於官網下單門市取貨者 當日到店取貨且在門市不限消費金額現折100 POS操作：輸入會員條碼→再輸入折扣碼【PICKUP100】</t>
-  </si>
-  <si>
     <t>2026/06/30郵件</t>
   </si>
   <si>
@@ -1336,9 +1327,6 @@
     <t>7/9-7/26</t>
   </si>
   <si>
-    <t>7/9-7/26 部分店櫃適用 一般會員/過路客滿3200贈玩總行李吊牌 VIP/SVIP滿2500贈玩總行李吊牌 左營新光店、台中漢神店、嘉義秀泰店、新台南FOCUS店 [image: image.png]</t>
-  </si>
-  <si>
     <t>台中漢神</t>
   </si>
   <si>
@@ -1348,37 +1336,75 @@
     <t>7/6-7/12</t>
   </si>
   <si>
-    <t>7/6-7/12 IP專賣店櫃獨家 消費DINOTAENG商品即贈DINOTAENG滑鼠墊 全館滿2500贈DINOTAENG手機鍊 [image: image.png]</t>
-  </si>
-  <si>
-    <t>7/13-7/26 IP專賣店櫃獨家 消費DINOTAENG商品即贈DINOTAENG手機支架 [image: image.png]</t>
-  </si>
-  <si>
-    <t>7/9-7/12</t>
-  </si>
-  <si>
     <t>會員專屬</t>
   </si>
   <si>
-    <t>情境說明 若於7/9-7/12 之間VIP/SVIP消費滿2500</t>
-  </si>
-  <si>
     <t>適用門市/通路</t>
   </si>
   <si>
-    <t>適用百貨 新莊宏匯/桃園台茂/桃園大江/桃園統領/新光中港/夢時代/新光左營</t>
+    <t>7/13-7/19</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>全館商品三件以上85折</t>
+    <t>08/10-08/23</t>
+  </si>
+  <si>
+    <t>滿2500贈袋鼠購物袋組 (不分會員) 滿3200贈玩總行李吊牌 (一般及非會員) 滿2500贈玩總行李吊牌 (SVIP及VIP)</t>
+  </si>
+  <si>
+    <t>滿2500贈烤焦KT絨毛吊飾 (不分會員) 滿3200贈玩總行李吊牌 (一般及非會員) 滿2500贈玩總行李吊牌 (SVIP及VIP)</t>
+  </si>
+  <si>
+    <t>08/10-08/16</t>
+  </si>
+  <si>
+    <t>08/10-08/16 門網同步 (IP正價店不適用) 全館三件85折、滿3800再折380</t>
+  </si>
+  <si>
+    <t>IP商品/當年度KOL聯名款/甜甜價/體驗價/組合價(包含買單件)*不列入三件折扣;但可湊滿額折價</t>
+  </si>
+  <si>
+    <t>08/17-08/30</t>
+  </si>
+  <si>
+    <t>08/21-08/24</t>
+  </si>
+  <si>
+    <t>08/24-09/13</t>
+  </si>
+  <si>
+    <t>IP專賣店活動 滿1800贈$150紅利金 (8/31、9/7、9/14匯入點數) 滿2500贈烤焦KT絨毛吊飾 (不分會員) 滿3200贈玩總行李吊牌 (一般及非會員) 滿2500贈玩總行李吊牌 (SVIP及VIP)</t>
+  </si>
+  <si>
+    <t>08/24-09/13</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>部分百貨提前開跑</t>
+    <t>買當周新品加倍贈紅利點數</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>7/13-7/19</t>
+    <t>08/17-09/13</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>08/17-08/30 春夏鞋款全館單件65折 (排除聯名款) 大碼商品全館單件85折</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>08/21-08/24 &amp; 08/28-08/30 門網同步加碼 精選泳裝單件39折</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/13-7/26 IP專賣店櫃獨家 消費DINOTAENG商品即贈DINOTAENG手機支架</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/6-7/12 IP專賣店櫃獨家 消費DINOTAENG商品即贈DINOTAENG滑鼠墊 全館滿2500贈DINOTAENG手機鍊</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/9-7/26 部分店櫃適用 一般會員/過路客滿3200贈玩總行李吊牌 VIP/SVIP滿2500贈玩總行李吊牌 左營新光店、台中漢神店、嘉義秀泰店、新台南FOCUS店</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1386,10 +1412,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="176" formatCode="m/d"/>
+    <numFmt numFmtId="181" formatCode="m&quot;月&quot;d&quot;日&quot;"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1414,13 +1441,6 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="微軟正黑體"/>
-      <family val="2"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FFFF0000"/>
       <name val="微軟正黑體"/>
       <family val="2"/>
       <charset val="136"/>
@@ -1556,14 +1576,134 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="181" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="30">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDEEBF7"/>
+          <bgColor rgb="FFDEEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE4D6"/>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEDEDED"/>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF2F2F2"/>
+          <bgColor rgb="FFF2F2F2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEDEDED"/>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2EFDA"/>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2EFDA"/>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2EFDA"/>
+          <bgColor rgb="FFE2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFBDD7EE"/>
+          <bgColor rgb="FFBDD7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDEEBF7"/>
+          <bgColor rgb="FFDEEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE4D6"/>
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1896,12 +2036,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I997"/>
+  <dimension ref="A1:I982"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="6" style="4" customWidth="1"/>
     <col min="3" max="4" width="16" style="4" customWidth="1"/>
-    <col min="5" max="5" width="61.7109375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="255.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22" style="4" customWidth="1"/>
     <col min="7" max="7" width="14" style="4" customWidth="1"/>
     <col min="8" max="8" width="62.7109375" style="4" customWidth="1"/>
@@ -1927,7 +2067,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>5</v>
@@ -5909,7 +6049,7 @@
         <v>396</v>
       </c>
       <c r="I138" s="15" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="139" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6151,14 +6291,14 @@
       <c r="B147" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C147" s="16" t="s">
-        <v>426</v>
+      <c r="C147" s="15" t="s">
+        <v>424</v>
       </c>
       <c r="D147" s="15" t="s">
         <v>95</v>
       </c>
       <c r="E147" s="15" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F147" s="15" t="s">
         <v>18</v>
@@ -6167,10 +6307,10 @@
         <v>19</v>
       </c>
       <c r="H147" s="15" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="I147" s="15" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="148" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6180,7 +6320,7 @@
       <c r="B148" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C148" s="16" t="s">
+      <c r="C148" s="15" t="s">
         <v>418</v>
       </c>
       <c r="D148" s="15" t="s">
@@ -6196,10 +6336,10 @@
         <v>19</v>
       </c>
       <c r="H148" s="15" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="I148" s="15" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="149" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6209,7 +6349,7 @@
       <c r="B149" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C149" s="16" t="s">
+      <c r="C149" s="15" t="s">
         <v>420</v>
       </c>
       <c r="D149" s="15" t="s">
@@ -6238,14 +6378,14 @@
       <c r="B150" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C150" s="16" t="s">
-        <v>431</v>
+      <c r="C150" s="15" t="s">
+        <v>429</v>
       </c>
       <c r="D150" s="15" t="s">
         <v>397</v>
       </c>
       <c r="E150" s="15" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="F150" s="15" t="s">
         <v>12</v>
@@ -6257,7 +6397,7 @@
         <v>13</v>
       </c>
       <c r="I150" s="15" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="151" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6267,14 +6407,14 @@
       <c r="B151" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C151" s="16" t="s">
-        <v>431</v>
+      <c r="C151" s="15" t="s">
+        <v>429</v>
       </c>
       <c r="D151" s="15" t="s">
         <v>32</v>
       </c>
       <c r="E151" s="15" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="F151" s="15" t="s">
         <v>118</v>
@@ -6286,7 +6426,7 @@
         <v>13</v>
       </c>
       <c r="I151" s="15" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="152" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6296,26 +6436,26 @@
       <c r="B152" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C152" s="16" t="s">
-        <v>423</v>
+      <c r="C152" s="15" t="s">
+        <v>415</v>
       </c>
       <c r="D152" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E152" s="15" t="s">
-        <v>450</v>
+        <v>416</v>
       </c>
       <c r="F152" s="15" t="s">
-        <v>451</v>
+        <v>12</v>
       </c>
       <c r="G152" s="15" t="s">
         <v>19</v>
       </c>
       <c r="H152" s="15" t="s">
-        <v>449</v>
+        <v>417</v>
       </c>
       <c r="I152" s="15" t="s">
-        <v>424</v>
+        <v>412</v>
       </c>
     </row>
     <row r="153" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6323,10 +6463,10 @@
         <v>2026</v>
       </c>
       <c r="B153" s="15" t="s">
-        <v>103</v>
-      </c>
-      <c r="C153" s="16" t="s">
-        <v>415</v>
+        <v>122</v>
+      </c>
+      <c r="C153" s="15" t="s">
+        <v>441</v>
       </c>
       <c r="D153" s="15" t="s">
         <v>22</v>
@@ -6340,11 +6480,9 @@
       <c r="G153" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="H153" s="15" t="s">
-        <v>417</v>
-      </c>
+      <c r="H153" s="15"/>
       <c r="I153" s="15" t="s">
-        <v>412</v>
+        <v>432</v>
       </c>
     </row>
     <row r="154" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6354,14 +6492,14 @@
       <c r="B154" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="C154" s="16" t="s">
-        <v>452</v>
+      <c r="C154" s="15" t="s">
+        <v>434</v>
       </c>
       <c r="D154" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="E154" s="16" t="s">
-        <v>416</v>
+        <v>397</v>
+      </c>
+      <c r="E154" s="15" t="s">
+        <v>457</v>
       </c>
       <c r="F154" s="15" t="s">
         <v>12</v>
@@ -6369,9 +6507,11 @@
       <c r="G154" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="H154" s="15"/>
+      <c r="H154" s="15" t="s">
+        <v>13</v>
+      </c>
       <c r="I154" s="15" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="155" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6382,13 +6522,13 @@
         <v>122</v>
       </c>
       <c r="C155" s="15" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D155" s="15" t="s">
-        <v>397</v>
+        <v>95</v>
       </c>
       <c r="E155" s="15" t="s">
-        <v>444</v>
+        <v>458</v>
       </c>
       <c r="F155" s="15" t="s">
         <v>12</v>
@@ -6400,7 +6540,7 @@
         <v>13</v>
       </c>
       <c r="I155" s="15" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="156" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6411,83 +6551,80 @@
         <v>122</v>
       </c>
       <c r="C156" s="15" t="s">
-        <v>442</v>
+        <v>435</v>
       </c>
       <c r="D156" s="15" t="s">
         <v>95</v>
       </c>
       <c r="E156" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="F156" s="15" t="s">
+        <v>436</v>
+      </c>
+      <c r="G156" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="H156" s="15" t="s">
+        <v>437</v>
+      </c>
+      <c r="I156" s="15" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B157" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C157" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D157" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="E157" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="F157" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G157" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H157" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="I157" s="4" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="D158" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E158" s="4" t="s">
         <v>443</v>
       </c>
-      <c r="F156" s="15" t="s">
+      <c r="F158" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G156" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="H156" s="15" t="s">
+      <c r="G158" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H158" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="I156" s="15" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="157" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="15">
-        <v>2026</v>
-      </c>
-      <c r="B157" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="C157" s="15" t="s">
-        <v>445</v>
-      </c>
-      <c r="D157" s="15" t="s">
-        <v>446</v>
-      </c>
-      <c r="E157" s="15" t="s">
-        <v>447</v>
-      </c>
-      <c r="F157" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="G157" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="H157" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="I157" s="15" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="158" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="15">
-        <v>2026</v>
-      </c>
-      <c r="B158" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="C158" s="15" t="s">
-        <v>438</v>
-      </c>
-      <c r="D158" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="E158" s="15" t="s">
-        <v>439</v>
-      </c>
-      <c r="F158" s="15" t="s">
-        <v>440</v>
-      </c>
-      <c r="G158" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="H158" s="15" t="s">
-        <v>441</v>
-      </c>
-      <c r="I158" s="15" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="159" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6498,13 +6635,13 @@
         <v>135</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>137</v>
+        <v>452</v>
       </c>
       <c r="D159" s="4" t="s">
-        <v>390</v>
+        <v>95</v>
       </c>
       <c r="E159" s="4" t="s">
-        <v>391</v>
+        <v>444</v>
       </c>
       <c r="F159" s="4" t="s">
         <v>12</v>
@@ -6513,10 +6650,7 @@
         <v>19</v>
       </c>
       <c r="H159" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="I159" s="4" t="s">
-        <v>392</v>
+        <v>13</v>
       </c>
     </row>
     <row r="160" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6527,13 +6661,13 @@
         <v>135</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>137</v>
+        <v>445</v>
       </c>
       <c r="D160" s="4" t="s">
-        <v>390</v>
+        <v>16</v>
       </c>
       <c r="E160" s="4" t="s">
-        <v>391</v>
+        <v>446</v>
       </c>
       <c r="F160" s="4" t="s">
         <v>12</v>
@@ -6542,13 +6676,10 @@
         <v>19</v>
       </c>
       <c r="H160" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="I160" s="4" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="161" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="4">
         <v>2026</v>
       </c>
@@ -6556,42 +6687,114 @@
         <v>135</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>137</v>
+        <v>448</v>
       </c>
       <c r="D161" s="4" t="s">
-        <v>390</v>
+        <v>22</v>
       </c>
       <c r="E161" s="4" t="s">
-        <v>434</v>
+        <v>455</v>
       </c>
       <c r="F161" s="4" t="s">
         <v>12</v>
       </c>
       <c r="G161" s="4" t="s">
-        <v>19</v>
+        <v>115</v>
       </c>
       <c r="H161" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="I161" s="4" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="162" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C162" s="16" t="s">
+        <v>454</v>
+      </c>
+      <c r="D162" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="E162" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="F162" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G162" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H162" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C163" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D163" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E163" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="F163" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G163" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="H163" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C164" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="D164" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E164" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="F164" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G164" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H164" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -7398,21 +7601,6 @@
     <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:I151">
     <sortState ref="A2:I164">
@@ -7420,77 +7608,77 @@
     </sortState>
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="14" priority="1" stopIfTrue="1" operator="equal">
       <formula>"調整後"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="13" priority="2" stopIfTrue="1" operator="equal">
       <formula>"再次調整"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="12" priority="3" stopIfTrue="1" operator="equal">
       <formula>"延長"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="11" priority="4" stopIfTrue="1" operator="equal">
       <formula>"再次延長"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="10" priority="5" stopIfTrue="1" operator="equal">
       <formula>"加碼"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="9" priority="6" stopIfTrue="1" operator="equal">
       <formula>"獨家加碼"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="8" priority="7" stopIfTrue="1" operator="equal">
       <formula>"搶先開跑"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="7" priority="8" stopIfTrue="1" operator="equal">
       <formula>"取消"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="6" priority="9" stopIfTrue="1" operator="equal">
       <formula>"補充"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="5" priority="10" stopIfTrue="1" operator="equal">
       <formula>"長期"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="4" priority="11" stopIfTrue="1" operator="equal">
       <formula>"日期調整"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="3" priority="12" stopIfTrue="1" operator="equal">
       <formula>"系統調整"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="2" priority="13" stopIfTrue="1" operator="equal">
       <formula>"原訂(後改)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="1" priority="14" stopIfTrue="1" operator="equal">
       <formula>"原訂(後延長)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G997">
+  <conditionalFormatting sqref="G2:G982">
     <cfRule type="cellIs" dxfId="0" priority="15" stopIfTrue="1" operator="equal">
       <formula>"原訂(後取消)"</formula>
     </cfRule>

</xml_diff>